<commit_message>
Para análise: Atualização dos Slides e a Planilha de Requisitos
</commit_message>
<xml_diff>
--- a/Documentos/Planilha de Requisitos - WHIS{KEY}.xlsx
+++ b/Documentos/Planilha de Requisitos - WHIS{KEY}.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83966574-C2F9-4921-950D-8163E7881883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6622D939-2C9F-4AE8-80F5-E739A8873DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos Projeto" sheetId="1" r:id="rId1"/>
-    <sheet name="Planilha Requisitos SP2" sheetId="3" r:id="rId2"/>
+    <sheet name="Planilha Requisitos SP2 (2)" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requisitos Projeto'!#REF!</definedName>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="138">
   <si>
     <t>Planilha de requisitos</t>
   </si>
@@ -448,6 +448,9 @@
   </si>
   <si>
     <t>SELECIONAR MINI SPRINT (A -D)</t>
+  </si>
+  <si>
+    <t>SPRINT</t>
   </si>
 </sst>
 </file>
@@ -461,7 +464,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -676,8 +679,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="8" tint="-0.249977111117893"/>
+      <name val="Univers"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="44">
+  <fills count="45">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -923,8 +933,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -1190,6 +1206,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1240,7 +1265,7 @@
     <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1380,16 +1405,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1405,9 +1436,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="43" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1428,17 +1456,26 @@
     <xf numFmtId="0" fontId="0" fillId="43" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="35" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="35" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="47">
@@ -1706,15 +1743,15 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="16"/>
-        <color theme="8" tint="-0.249977111117893"/>
+        <color rgb="FF2E653D"/>
         <name val="Univers"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FFDFE3E5"/>
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2750,7 +2787,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>378</c:v>
+                  <c:v>294</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>93</c:v>
@@ -3052,379 +3089,6 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="107"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="7"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                  <a:prstClr val="black">
-                    <a:alpha val="40000"/>
-                  </a:prstClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="pt-BR"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="stacked"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Requisitos Projeto'!$E$85</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Progresso</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="34925" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="lt1">
-                        <a:lumMod val="85000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="pt-BR"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="t"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="lt1">
-                          <a:lumMod val="95000"/>
-                          <a:alpha val="54000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Requisitos Projeto'!$D$86:$D$89</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>TOTAL</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v> SP1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>SP2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>SP3</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Requisitos Projeto'!$E$86:$E$89</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>378</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>285</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>84</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8DA0-4863-B23E-317C9A233EC6}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="t"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="1488008272"/>
-        <c:axId val="1488007312"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="1488008272"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:lumMod val="95000"/>
-                <a:alpha val="10000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="pt-BR"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1488007312"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1488007312"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                  <a:alpha val="10000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="pt-BR"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1488008272"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="zero"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:gradFill flip="none" rotWithShape="1">
-      <a:gsLst>
-        <a:gs pos="0">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:gs>
-        <a:gs pos="100000">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="85000"/>
-            <a:lumOff val="15000"/>
-          </a:schemeClr>
-        </a:gs>
-      </a:gsLst>
-      <a:path path="circle">
-        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-      </a:path>
-      <a:tileRect/>
-    </a:gradFill>
-    <a:ln>
-      <a:noFill/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="pt-BR"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
       <c14:style val="102"/>
     </mc:Choice>
     <mc:Fallback>
@@ -3510,7 +3174,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Planilha Requisitos SP2'!$D$59</c:f>
+              <c:f>'Planilha Requisitos SP2 (2)'!$D$59</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3595,7 +3259,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Planilha Requisitos SP2'!$C$60:$C$64</c:f>
+              <c:f>'Planilha Requisitos SP2 (2)'!$C$60:$C$64</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3618,7 +3282,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Planilha Requisitos SP2'!$D$60:$D$64</c:f>
+              <c:f>'Planilha Requisitos SP2 (2)'!$D$60:$D$64</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3643,7 +3307,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7237-4D56-B87A-12053D384841}"/>
+              <c16:uniqueId val="{00000000-0909-4A96-8281-E7857BEB5F3A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3866,12 +3530,6 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="18">
-  <a:schemeClr val="accent5"/>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4903,516 +4561,20 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="233">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:gradFill flip="none" rotWithShape="1">
-        <a:gsLst>
-          <a:gs pos="0">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="65000"/>
-              <a:lumOff val="35000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="100000">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="85000"/>
-              <a:lumOff val="15000"/>
-            </a:schemeClr>
-          </a:gs>
-        </a:gsLst>
-        <a:path path="circle">
-          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-        </a:path>
-        <a:tileRect/>
-      </a:gradFill>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="34925" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="5000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="95000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
-    </cs:defRPr>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>807041</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>115769</xdr:rowOff>
+      <xdr:colOff>803935</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>336294</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>9098256</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>28854</xdr:rowOff>
+      <xdr:colOff>9095150</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>241096</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5440,15 +4602,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>252704</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>77756</xdr:rowOff>
+      <xdr:colOff>329711</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>36635</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>5229030</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>416921</xdr:rowOff>
+      <xdr:colOff>4707547</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>274759</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5463,7 +4625,7 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill>
+      <xdr:blipFill rotWithShape="1">
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
@@ -5471,14 +4633,15 @@
             </a:ext>
           </a:extLst>
         </a:blip>
+        <a:srcRect l="7805" t="11386" r="4222" b="25275"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="547113" y="77756"/>
-          <a:ext cx="4976326" cy="2555892"/>
+          <a:off x="622788" y="293077"/>
+          <a:ext cx="4377836" cy="1630240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5490,15 +4653,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1060331</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>323491</xdr:rowOff>
+      <xdr:colOff>1081037</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>80188</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>3726114</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>179716</xdr:rowOff>
+      <xdr:colOff>3746820</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>317415</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5527,139 +4690,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1347878" y="24423538"/>
-          <a:ext cx="2665783" cy="1365848"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1060331</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>323491</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2665783" cy="1380225"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagem 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C78241BD-8C3B-4D64-A7F2-932796059DF4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1354740" y="23114218"/>
-          <a:ext cx="2665783" cy="1380225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>850446</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>9523</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>9089571</xdr:colOff>
-      <xdr:row>102</xdr:row>
-      <xdr:rowOff>108856</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Gráfico 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF565E72-3D61-7106-2714-A92222A76D96}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>911680</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>299358</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2435680</xdr:colOff>
-      <xdr:row>81</xdr:row>
-      <xdr:rowOff>326418</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagem 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0DD653E-4818-4675-96AC-89E8068EFB51}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1197430" y="31854322"/>
-          <a:ext cx="1524000" cy="789060"/>
+          <a:off x="1366787" y="23606938"/>
+          <a:ext cx="2665783" cy="1380227"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5688,10 +4720,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagem 4">
+        <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E23EB46-B6B8-4847-A72B-B0BB02B50CAB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5EF6979A-0C3B-4919-A75F-FAD8CD826860}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5714,7 +4746,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="320174" y="9921"/>
-          <a:ext cx="3230088" cy="1718469"/>
+          <a:ext cx="3230088" cy="1664494"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5738,14 +4770,16 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Gráfico 3">
+        <xdr:cNvPr id="3" name="Gráfico 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82AC63C1-FBC7-F782-50DE-92ADBA28BE7C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB9417DC-3A42-4BC7-A301-A55460AB6C08}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -5774,10 +4808,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Imagem 5">
+        <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DBDA498A-A2B3-45FE-A1FE-A3A4EA191BF7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21F1E4CE-D8E8-4A70-B26A-C8DDCFB16752}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5799,8 +4833,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4597783" y="9732690"/>
-          <a:ext cx="1747444" cy="896137"/>
+          <a:off x="4597783" y="9682272"/>
+          <a:ext cx="1745439" cy="884678"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5814,15 +4848,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Inventory_List_Table" displayName="Inventory_List_Table" ref="B4:H57" headerRowDxfId="28" dataDxfId="27">
-  <autoFilter ref="B4:H57" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
-  </autoFilter>
+  <autoFilter ref="B4:H57" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:H53">
     <sortCondition ref="H5:H53"/>
   </sortState>
@@ -5839,28 +4865,28 @@
 IF(Inventory_List_Table[[#This Row],[Tamanho]]="GG",21,0)))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Prioridade" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SP3" dataDxfId="14" totalsRowDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SPRINT" dataDxfId="14" totalsRowDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DFEF5BB9-030F-49A9-A8A6-AC82E626FC0E}" name="Tabela3" displayName="Tabela3" ref="A9:G36" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{593759BF-DCCE-4953-BECF-ADBBD89465DB}" name="Tabela33" displayName="Tabela33" ref="A9:G36" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1A52E22D-2CF6-4D98-A87D-1AA662C3121E}" name="Requisito" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{764E5F42-356E-4F61-BE66-B2F069497952}" name="Descrição" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{E7CD2CCE-8CD7-4445-AD40-E29C3D0E42D4}" name="Classificação" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A86194DD-DD7C-44E4-A6F9-6B3373149526}" name="Tamanho" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{AC635265-1FFE-43F6-B229-3E1FC0B65C8F}" name="Tam(#)" dataDxfId="6">
-      <calculatedColumnFormula>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{3ABB08E5-2C9A-4690-AF45-A43E6CBFA44A}" name="Requisito" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{39D6DADD-7441-407B-9F79-BAEBC33D5AC6}" name="Descrição" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{073C81CA-2398-4795-BB59-552ED9C428B9}" name="Classificação" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{72027A84-3E52-4152-8205-086C0FF73974}" name="Tamanho" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{3E797D67-7B5C-4095-8F33-07FC6B730416}" name="Tam(#)" dataDxfId="6">
+      <calculatedColumnFormula>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{39BC7F66-6245-4FEC-82DE-24821B3D7E96}" name="Prioridade" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{38070FD4-3ECF-4C86-B9E2-D32D410C7F06}" name="Sprint" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{88DE098E-9146-48CA-B3AD-2D8D988F38DB}" name="Prioridade" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{242D26B9-0ED8-43C2-9CAB-8EFFEC9D3DFD}" name="Sprint" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6097,26 +5123,26 @@
     </row>
     <row r="2" spans="1:9" ht="110.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
       <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:9" ht="45.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:9" s="4" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6140,7 +5166,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="34" t="s">
-        <v>95</v>
+        <v>137</v>
       </c>
       <c r="I4" s="24"/>
     </row>
@@ -6596,19 +5622,19 @@
     </row>
     <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23"/>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="56">
         <f>IF(Inventory_List_Table[[#This Row],[Tamanho]]="PP",3,
 IF(Inventory_List_Table[[#This Row],[Tamanho]]="P",5,
 IF(Inventory_List_Table[[#This Row],[Tamanho]]="M",8,
@@ -6616,10 +5642,10 @@
 IF(Inventory_List_Table[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="54">
         <v>1</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="54" t="s">
         <v>47</v>
       </c>
       <c r="I20" s="23"/>
@@ -7759,10 +6785,10 @@
       <c r="F61" s="47" t="s">
         <v>115</v>
       </c>
-      <c r="G61" s="59" t="s">
+      <c r="G61" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="H61" s="60"/>
+      <c r="H61" s="62"/>
       <c r="I61" s="23"/>
     </row>
     <row r="62" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7777,13 +6803,14 @@
         <v>378</v>
       </c>
       <c r="F62" s="15">
-        <f>SUM(Inventory_List_Table[Tam('#)])</f>
-        <v>378</v>
-      </c>
-      <c r="G62" s="55">
-        <v>0</v>
-      </c>
-      <c r="H62" s="56"/>
+        <f>SUM(Inventory_List_Table[Tam('#)])-E65</f>
+        <v>294</v>
+      </c>
+      <c r="G62" s="59">
+        <f>E62-F62</f>
+        <v>84</v>
+      </c>
+      <c r="H62" s="60"/>
       <c r="I62" s="23"/>
     </row>
     <row r="63" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7801,10 +6828,10 @@
         <f>SUM(F5:F19)</f>
         <v>93</v>
       </c>
-      <c r="G63" s="57">
+      <c r="G63" s="59">
         <v>0</v>
       </c>
-      <c r="H63" s="58"/>
+      <c r="H63" s="60"/>
       <c r="I63" s="23"/>
     </row>
     <row r="64" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7822,11 +6849,11 @@
         <f>SUM(F40,F46,F45,F44,F42,F41,F20:F39,F43)</f>
         <v>201</v>
       </c>
-      <c r="G64" s="57">
+      <c r="G64" s="59">
         <f>E64-F64</f>
         <v>0</v>
       </c>
-      <c r="H64" s="58"/>
+      <c r="H64" s="60"/>
       <c r="I64" s="23"/>
     </row>
     <row r="65" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7843,11 +6870,11 @@
       <c r="F65" s="11">
         <v>0</v>
       </c>
-      <c r="G65" s="57">
+      <c r="G65" s="59">
         <f>E65-F65</f>
         <v>84</v>
       </c>
-      <c r="H65" s="58"/>
+      <c r="H65" s="60"/>
       <c r="I65" s="23"/>
     </row>
     <row r="66" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8039,302 +7066,231 @@
     </row>
     <row r="83" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="23"/>
-      <c r="B83" s="29"/>
-      <c r="C83" s="29"/>
-      <c r="D83" s="30"/>
-      <c r="E83" s="30"/>
-      <c r="F83" s="30"/>
-      <c r="G83" s="30"/>
-      <c r="H83" s="30"/>
-      <c r="I83" s="23"/>
+      <c r="B83" s="53"/>
+      <c r="C83" s="53"/>
+      <c r="D83" s="53"/>
+      <c r="E83" s="53"/>
+      <c r="F83" s="53"/>
+      <c r="G83" s="53"/>
+      <c r="H83" s="53"/>
+      <c r="I83" s="53"/>
     </row>
     <row r="84" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="23"/>
-      <c r="B84" s="29"/>
-      <c r="C84" s="29"/>
-      <c r="D84" s="30"/>
-      <c r="E84" s="30"/>
-      <c r="F84" s="30"/>
-      <c r="G84" s="30"/>
-      <c r="H84" s="30"/>
-      <c r="I84" s="23"/>
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
     </row>
     <row r="85" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="23"/>
-      <c r="B85" s="29"/>
-      <c r="C85" s="31"/>
-      <c r="D85" s="30"/>
-      <c r="E85" s="46" t="s">
-        <v>135</v>
-      </c>
-      <c r="F85" s="30"/>
-      <c r="G85" s="30"/>
-      <c r="H85" s="30"/>
-      <c r="I85" s="23"/>
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
     </row>
     <row r="86" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="23"/>
-      <c r="B86" s="29"/>
-      <c r="C86" s="29"/>
-      <c r="D86" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="E86" s="15">
-        <f>SUM(Inventory_List_Table[Tam('#)])</f>
-        <v>378</v>
-      </c>
-      <c r="F86" s="30"/>
-      <c r="G86" s="30"/>
-      <c r="H86" s="30"/>
-      <c r="I86" s="22"/>
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
     </row>
     <row r="87" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="23"/>
-      <c r="B87" s="29"/>
-      <c r="C87" s="29"/>
-      <c r="D87" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="E87" s="13">
-        <f>E86-F63</f>
-        <v>285</v>
-      </c>
-      <c r="F87" s="30"/>
-      <c r="G87" s="30"/>
-      <c r="H87" s="30"/>
-      <c r="I87" s="23"/>
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
     </row>
     <row r="88" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="23"/>
-      <c r="B88" s="29"/>
-      <c r="C88" s="29"/>
-      <c r="D88" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E88" s="13">
-        <f>E87-F64</f>
-        <v>84</v>
-      </c>
-      <c r="F88" s="30"/>
-      <c r="G88" s="30"/>
-      <c r="H88" s="30"/>
-      <c r="I88" s="23"/>
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
     </row>
     <row r="89" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="23"/>
-      <c r="B89" s="29"/>
-      <c r="C89" s="29"/>
-      <c r="D89" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E89" s="13">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="F89" s="30"/>
-      <c r="G89" s="30"/>
-      <c r="H89" s="30"/>
-      <c r="I89" s="24"/>
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
     </row>
     <row r="90" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="23"/>
-      <c r="B90" s="29"/>
-      <c r="C90" s="32"/>
-      <c r="D90" s="30"/>
-      <c r="E90" s="30"/>
-      <c r="F90" s="30"/>
-      <c r="G90" s="30"/>
-      <c r="H90" s="30"/>
-      <c r="I90" s="23"/>
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
     </row>
     <row r="91" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="23"/>
-      <c r="B91" s="29"/>
-      <c r="C91" s="33"/>
-      <c r="D91" s="30"/>
-      <c r="E91" s="30"/>
-      <c r="F91" s="30"/>
-      <c r="G91" s="30"/>
-      <c r="H91" s="30"/>
-      <c r="I91" s="23"/>
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
     </row>
     <row r="92" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="23"/>
-      <c r="B92" s="29"/>
-      <c r="C92" s="33"/>
-      <c r="D92" s="30"/>
-      <c r="E92" s="30"/>
-      <c r="F92" s="30"/>
-      <c r="G92" s="30"/>
-      <c r="H92" s="30"/>
-      <c r="I92" s="23"/>
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
     </row>
     <row r="93" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="23"/>
-      <c r="B93" s="29"/>
-      <c r="C93" s="29"/>
-      <c r="D93" s="30"/>
-      <c r="E93" s="30"/>
-      <c r="F93" s="30"/>
-      <c r="G93" s="30"/>
-      <c r="H93" s="30"/>
-      <c r="I93" s="23"/>
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
     </row>
     <row r="94" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="23"/>
-      <c r="B94" s="29"/>
-      <c r="C94" s="29"/>
-      <c r="D94" s="30"/>
-      <c r="E94" s="30"/>
-      <c r="F94" s="30"/>
-      <c r="G94" s="30"/>
-      <c r="H94" s="30"/>
-      <c r="I94" s="23"/>
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
     </row>
     <row r="95" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="23"/>
-      <c r="B95" s="29"/>
-      <c r="C95" s="29"/>
-      <c r="D95" s="30"/>
-      <c r="E95" s="30"/>
-      <c r="F95" s="30"/>
-      <c r="G95" s="30"/>
-      <c r="H95" s="30"/>
-      <c r="I95" s="23"/>
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
     </row>
     <row r="96" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="23"/>
-      <c r="B96" s="29"/>
-      <c r="C96" s="29"/>
-      <c r="D96" s="30"/>
-      <c r="E96" s="30"/>
-      <c r="F96" s="30"/>
-      <c r="G96" s="30"/>
-      <c r="H96" s="30"/>
-      <c r="I96" s="23"/>
-    </row>
-    <row r="97" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="23"/>
-      <c r="B97" s="29"/>
-      <c r="C97" s="29"/>
-      <c r="D97" s="30"/>
-      <c r="E97" s="30"/>
-      <c r="F97" s="30"/>
-      <c r="G97" s="30"/>
-      <c r="H97" s="30"/>
-      <c r="I97" s="23"/>
-    </row>
-    <row r="98" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="23"/>
-      <c r="B98" s="29"/>
-      <c r="C98" s="29"/>
-      <c r="D98" s="30"/>
-      <c r="E98" s="30"/>
-      <c r="F98" s="30"/>
-      <c r="G98" s="30"/>
-      <c r="H98" s="30"/>
-      <c r="I98" s="23"/>
-    </row>
-    <row r="99" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="23"/>
-      <c r="B99" s="29"/>
-      <c r="C99" s="29"/>
-      <c r="D99" s="30"/>
-      <c r="E99" s="30"/>
-      <c r="F99" s="30"/>
-      <c r="G99" s="30"/>
-      <c r="H99" s="30"/>
-      <c r="I99" s="23"/>
-    </row>
-    <row r="100" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="23"/>
-      <c r="B100" s="29"/>
-      <c r="C100" s="29"/>
-      <c r="D100" s="30"/>
-      <c r="E100" s="30"/>
-      <c r="F100" s="30"/>
-      <c r="G100" s="30"/>
-      <c r="H100" s="30"/>
-      <c r="I100" s="23"/>
-    </row>
-    <row r="101" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="23"/>
-      <c r="B101" s="29"/>
-      <c r="C101" s="29"/>
-      <c r="D101" s="30"/>
-      <c r="E101" s="30"/>
-      <c r="F101" s="30"/>
-      <c r="G101" s="30"/>
-      <c r="H101" s="30"/>
-      <c r="I101" s="23"/>
-    </row>
-    <row r="102" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="23"/>
-      <c r="B102" s="29"/>
-      <c r="C102" s="29"/>
-      <c r="D102" s="30"/>
-      <c r="E102" s="30"/>
-      <c r="F102" s="30"/>
-      <c r="G102" s="30"/>
-      <c r="H102" s="30"/>
-      <c r="I102" s="23"/>
-    </row>
-    <row r="103" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="23"/>
-      <c r="B103" s="29"/>
-      <c r="C103" s="29"/>
-      <c r="D103" s="30"/>
-      <c r="E103" s="30"/>
-      <c r="F103" s="30"/>
-      <c r="G103" s="30"/>
-      <c r="H103" s="30"/>
-      <c r="I103" s="23"/>
-    </row>
-    <row r="104" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="23"/>
-      <c r="B104" s="29"/>
-      <c r="C104" s="29"/>
-      <c r="D104" s="30"/>
-      <c r="E104" s="30"/>
-      <c r="F104" s="30"/>
-      <c r="G104" s="30"/>
-      <c r="H104" s="30"/>
-      <c r="I104" s="23"/>
-    </row>
-    <row r="105" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="23"/>
-      <c r="B105" s="29"/>
-      <c r="C105" s="29"/>
-      <c r="D105" s="30"/>
-      <c r="E105" s="30"/>
-      <c r="F105" s="30"/>
-      <c r="G105" s="30"/>
-      <c r="H105" s="30"/>
-      <c r="I105" s="23"/>
-    </row>
-    <row r="106" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="23"/>
-      <c r="B106" s="23"/>
-      <c r="C106" s="23"/>
-      <c r="D106" s="23"/>
-      <c r="E106" s="23"/>
-      <c r="F106" s="23"/>
-      <c r="G106" s="23"/>
-      <c r="H106" s="23"/>
-      <c r="I106" s="23"/>
-    </row>
-    <row r="107" spans="1:9" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="23"/>
-      <c r="B107" s="23"/>
-      <c r="C107" s="23"/>
-      <c r="D107" s="23"/>
-      <c r="E107" s="23"/>
-      <c r="F107" s="23"/>
-      <c r="G107" s="23"/>
-      <c r="H107" s="23"/>
-      <c r="I107" s="23"/>
-    </row>
-    <row r="108" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+    </row>
+    <row r="97" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+    </row>
+    <row r="98" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+    </row>
+    <row r="99" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+    </row>
+    <row r="100" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+    </row>
+    <row r="101" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B101" s="3"/>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+    </row>
+    <row r="102" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B102" s="3"/>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+    </row>
+    <row r="103" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B103" s="3"/>
+      <c r="C103" s="3"/>
+      <c r="D103" s="3"/>
+      <c r="E103" s="3"/>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+    </row>
+    <row r="104" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B104" s="3"/>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3"/>
+      <c r="E104" s="3"/>
+      <c r="F104" s="3"/>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3"/>
+    </row>
+    <row r="105" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B105" s="3"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3"/>
+      <c r="E105" s="3"/>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+    </row>
+    <row r="106" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+      <c r="G106" s="3"/>
+      <c r="H106" s="3"/>
+    </row>
+    <row r="107" spans="2:8" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B107" s="3"/>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3"/>
+      <c r="E107" s="3"/>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+    </row>
+    <row r="108" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
@@ -8343,7 +7299,7 @@
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
     </row>
-    <row r="109" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
@@ -8352,7 +7308,7 @@
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
     </row>
-    <row r="110" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
@@ -8361,7 +7317,7 @@
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
     </row>
-    <row r="111" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
@@ -8370,7 +7326,7 @@
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
     </row>
-    <row r="112" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
@@ -9081,17 +8037,14 @@
       <formula>#REF!=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1141" yWindow="341" count="8">
+  <dataValidations xWindow="1141" yWindow="341" count="7">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nome do item nesta coluna" sqref="B4" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nível de estoque de cada item nesta coluna" sqref="G4" xr:uid="{00000000-0002-0000-0000-000007000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Esse é um valor de estoque column._x000a__x000a_O valor de estoque de cada item é automaticamente calculado nesta coluna." sqref="F4" xr:uid="{00000000-0002-0000-0000-000008000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira a quantidade em estoque de cada item nesta coluna" sqref="E4" xr:uid="{00000000-0002-0000-0000-000009000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o preço unitário de cada item nesta coluna" sqref="D4" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira uma descrição do item nesta coluna" sqref="C4" xr:uid="{00000000-0002-0000-0000-00000B000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Esta planilha controla o estoque dos itens listados na tabela de lista de estoque e possibilita realçar e sinalizar esses itens que já estão prontos para serem repostos. Itens descontinuados têm formatação Tachado e o texto &quot;sim&quot; na coluna correspondente." sqref="A1 I1 I86" xr:uid="{8F182C1C-C305-48BB-889F-2AD958D3312B}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira quantos dias faltam para realizar nova encomenda de cada item nesta coluna" sqref="H4" xr:uid="{00000000-0002-0000-0000-000006000000}">
-      <formula1>$H$5:$H$27</formula1>
-    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Esta planilha controla o estoque dos itens listados na tabela de lista de estoque e possibilita realçar e sinalizar esses itens que já estão prontos para serem repostos. Itens descontinuados têm formatação Tachado e o texto &quot;sim&quot; na coluna correspondente." sqref="A1 I1" xr:uid="{8F182C1C-C305-48BB-889F-2AD958D3312B}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9104,7 +8057,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85BC3CD0-F7F0-4C0E-883C-E32C34EA90D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D863DC5D-F27E-48D0-B8DF-8044B97C94FB}">
   <dimension ref="A1:G71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -9228,11 +8181,11 @@
         <v>19</v>
       </c>
       <c r="E10" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
       <c r="F10" s="39">
@@ -9256,11 +8209,11 @@
         <v>16</v>
       </c>
       <c r="E11" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F11" s="36">
@@ -9284,11 +8237,11 @@
         <v>16</v>
       </c>
       <c r="E12" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F12" s="39">
@@ -9312,11 +8265,11 @@
         <v>19</v>
       </c>
       <c r="E13" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
       <c r="F13" s="36">
@@ -9340,11 +8293,11 @@
         <v>10</v>
       </c>
       <c r="E14" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>3</v>
       </c>
       <c r="F14" s="39">
@@ -9368,11 +8321,11 @@
         <v>16</v>
       </c>
       <c r="E15" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F15" s="36">
@@ -9396,11 +8349,11 @@
         <v>29</v>
       </c>
       <c r="E16" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F16" s="39">
@@ -9424,11 +8377,11 @@
         <v>29</v>
       </c>
       <c r="E17" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F17" s="36">
@@ -9452,11 +8405,11 @@
         <v>16</v>
       </c>
       <c r="E18" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F18" s="39">
@@ -9480,11 +8433,11 @@
         <v>19</v>
       </c>
       <c r="E19" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
       <c r="F19" s="36">
@@ -9508,11 +8461,11 @@
         <v>29</v>
       </c>
       <c r="E20" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F20" s="39">
@@ -9536,11 +8489,11 @@
         <v>16</v>
       </c>
       <c r="E21" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F21" s="36">
@@ -9564,11 +8517,11 @@
         <v>16</v>
       </c>
       <c r="E22" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F22" s="39">
@@ -9592,11 +8545,11 @@
         <v>16</v>
       </c>
       <c r="E23" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F23" s="36">
@@ -9620,11 +8573,11 @@
         <v>16</v>
       </c>
       <c r="E24" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F24" s="39">
@@ -9648,11 +8601,11 @@
         <v>29</v>
       </c>
       <c r="E25" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F25" s="36">
@@ -9676,11 +8629,11 @@
         <v>29</v>
       </c>
       <c r="E26" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F26" s="39">
@@ -9704,11 +8657,11 @@
         <v>29</v>
       </c>
       <c r="E27" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F27" s="36">
@@ -9732,11 +8685,11 @@
         <v>29</v>
       </c>
       <c r="E28" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F28" s="39">
@@ -9760,11 +8713,11 @@
         <v>29</v>
       </c>
       <c r="E29" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F29" s="36">
@@ -9788,11 +8741,11 @@
         <v>16</v>
       </c>
       <c r="E30" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F30" s="39">
@@ -9816,11 +8769,11 @@
         <v>10</v>
       </c>
       <c r="E31" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>3</v>
       </c>
       <c r="F31" s="36">
@@ -9844,11 +8797,11 @@
         <v>19</v>
       </c>
       <c r="E32" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
       <c r="F32" s="39">
@@ -9872,11 +8825,11 @@
         <v>19</v>
       </c>
       <c r="E33" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>13</v>
       </c>
       <c r="F33" s="36">
@@ -9900,11 +8853,11 @@
         <v>16</v>
       </c>
       <c r="E34" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>8</v>
       </c>
       <c r="F34" s="39">
@@ -9928,11 +8881,11 @@
         <v>29</v>
       </c>
       <c r="E35" s="38">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F35" s="36">
@@ -9956,11 +8909,11 @@
         <v>29</v>
       </c>
       <c r="E36" s="41">
-        <f>IF(Tabela3[[#This Row],[Tamanho]]="PP",3,
-IF(Tabela3[[#This Row],[Tamanho]]="P",5,
-IF(Tabela3[[#This Row],[Tamanho]]="M",8,
-IF(Tabela3[[#This Row],[Tamanho]]="G",13,
-IF(Tabela3[[#This Row],[Tamanho]]="GG",21,0)))))</f>
+        <f>IF(Tabela33[[#This Row],[Tamanho]]="PP",3,
+IF(Tabela33[[#This Row],[Tamanho]]="P",5,
+IF(Tabela33[[#This Row],[Tamanho]]="M",8,
+IF(Tabela33[[#This Row],[Tamanho]]="G",13,
+IF(Tabela33[[#This Row],[Tamanho]]="GG",21,0)))))</f>
         <v>5</v>
       </c>
       <c r="F36" s="39">
@@ -9971,89 +8924,89 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="62"/>
-      <c r="B37" s="62"/>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
+      <c r="A37" s="71"/>
+      <c r="B37" s="71"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="63"/>
+      <c r="F37" s="63"/>
+      <c r="G37" s="63"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="62"/>
-      <c r="B38" s="62"/>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
+      <c r="A38" s="71"/>
+      <c r="B38" s="71"/>
+      <c r="C38" s="63"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="63"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="63"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="62"/>
-      <c r="B39" s="62"/>
-      <c r="C39" s="61"/>
-      <c r="D39" s="61"/>
-      <c r="E39" s="61"/>
-      <c r="F39" s="61"/>
-      <c r="G39" s="61"/>
+      <c r="A39" s="71"/>
+      <c r="B39" s="71"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
+      <c r="E39" s="63"/>
+      <c r="F39" s="63"/>
+      <c r="G39" s="63"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="62"/>
-      <c r="B40" s="62"/>
-      <c r="C40" s="61"/>
-      <c r="D40" s="61"/>
-      <c r="E40" s="61"/>
-      <c r="F40" s="61"/>
-      <c r="G40" s="61"/>
+      <c r="A40" s="71"/>
+      <c r="B40" s="71"/>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="63"/>
+      <c r="F40" s="63"/>
+      <c r="G40" s="63"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="62"/>
-      <c r="B41" s="62"/>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
+      <c r="A41" s="71"/>
+      <c r="B41" s="71"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="62"/>
-      <c r="B42" s="62"/>
-      <c r="C42" s="61"/>
-      <c r="D42" s="61"/>
-      <c r="E42" s="61"/>
-      <c r="F42" s="61"/>
-      <c r="G42" s="61"/>
+      <c r="A42" s="71"/>
+      <c r="B42" s="71"/>
+      <c r="C42" s="63"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="63"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="63"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="62"/>
-      <c r="B43" s="62"/>
-      <c r="C43" s="61"/>
-      <c r="D43" s="61"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="61"/>
-      <c r="G43" s="61"/>
+      <c r="A43" s="71"/>
+      <c r="B43" s="71"/>
+      <c r="C43" s="63"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="63"/>
+      <c r="F43" s="63"/>
+      <c r="G43" s="63"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="62"/>
-      <c r="B44" s="62"/>
-      <c r="C44" s="61"/>
-      <c r="D44" s="61"/>
-      <c r="E44" s="61"/>
-      <c r="F44" s="61"/>
-      <c r="G44" s="61"/>
+      <c r="A44" s="71"/>
+      <c r="B44" s="71"/>
+      <c r="C44" s="63"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="63"/>
+      <c r="F44" s="63"/>
+      <c r="G44" s="63"/>
     </row>
     <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="62"/>
-      <c r="B45" s="62"/>
-      <c r="C45" s="61"/>
-      <c r="D45" s="61"/>
-      <c r="E45" s="61"/>
-      <c r="F45" s="61"/>
-      <c r="G45" s="61"/>
+      <c r="A45" s="71"/>
+      <c r="B45" s="71"/>
+      <c r="C45" s="63"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="63"/>
+      <c r="F45" s="63"/>
+      <c r="G45" s="63"/>
     </row>
     <row r="46" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="62"/>
-      <c r="B46" s="62"/>
+      <c r="A46" s="71"/>
+      <c r="B46" s="71"/>
       <c r="C46" s="30"/>
       <c r="D46" s="12" t="s">
         <v>117</v>
@@ -10061,14 +9014,14 @@
       <c r="E46" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="F46" s="71" t="s">
+      <c r="F46" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="G46" s="72"/>
+      <c r="G46" s="73"/>
     </row>
     <row r="47" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="62"/>
-      <c r="B47" s="62"/>
+      <c r="A47" s="71"/>
+      <c r="B47" s="71"/>
       <c r="C47" s="14" t="s">
         <v>112</v>
       </c>
@@ -10080,15 +9033,15 @@
         <f>SUM(E48:E51)</f>
         <v>201</v>
       </c>
-      <c r="F47" s="55">
+      <c r="F47" s="74">
         <f>D47-E47</f>
         <v>0</v>
       </c>
-      <c r="G47" s="56"/>
+      <c r="G47" s="75"/>
     </row>
     <row r="48" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="62"/>
-      <c r="B48" s="62"/>
+      <c r="A48" s="71"/>
+      <c r="B48" s="71"/>
       <c r="C48" s="14" t="s">
         <v>123</v>
       </c>
@@ -10100,14 +9053,14 @@
         <f>SUM(E10:E11,E14,E24,E25)</f>
         <v>37</v>
       </c>
-      <c r="F48" s="57">
+      <c r="F48" s="59">
         <v>0</v>
       </c>
-      <c r="G48" s="58"/>
+      <c r="G48" s="60"/>
     </row>
     <row r="49" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="62"/>
-      <c r="B49" s="62"/>
+      <c r="A49" s="71"/>
+      <c r="B49" s="71"/>
       <c r="C49" s="14" t="s">
         <v>120</v>
       </c>
@@ -10119,15 +9072,15 @@
         <f>SUM(E12,E13,E20,E21,E22,E27,E28,E29)</f>
         <v>57</v>
       </c>
-      <c r="F49" s="57">
+      <c r="F49" s="59">
         <f>D49-E49</f>
         <v>0</v>
       </c>
-      <c r="G49" s="58"/>
+      <c r="G49" s="60"/>
     </row>
     <row r="50" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="62"/>
-      <c r="B50" s="62"/>
+      <c r="A50" s="71"/>
+      <c r="B50" s="71"/>
       <c r="C50" s="14" t="s">
         <v>122</v>
       </c>
@@ -10139,15 +9092,15 @@
         <f>SUM(E15,E17,E18,E19,E26,E30,E31,E32)</f>
         <v>63</v>
       </c>
-      <c r="F50" s="57">
+      <c r="F50" s="59">
         <f>D50-E50</f>
         <v>0</v>
       </c>
-      <c r="G50" s="58"/>
+      <c r="G50" s="60"/>
     </row>
     <row r="51" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="62"/>
-      <c r="B51" s="62"/>
+      <c r="A51" s="71"/>
+      <c r="B51" s="71"/>
       <c r="C51" s="14" t="s">
         <v>121</v>
       </c>
@@ -10159,91 +9112,91 @@
         <f>SUM(E16,E23,E34,E35,E36,E33)</f>
         <v>44</v>
       </c>
-      <c r="F51" s="57">
+      <c r="F51" s="59">
         <f>D51-E51</f>
         <v>0</v>
       </c>
-      <c r="G51" s="58"/>
+      <c r="G51" s="60"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="62"/>
-      <c r="B52" s="62"/>
-      <c r="C52" s="69"/>
-      <c r="D52" s="69"/>
-      <c r="E52" s="69"/>
+      <c r="A52" s="71"/>
+      <c r="B52" s="71"/>
+      <c r="C52" s="76"/>
+      <c r="D52" s="76"/>
+      <c r="E52" s="76"/>
       <c r="F52" s="48"/>
       <c r="G52" s="48"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="62"/>
-      <c r="B53" s="62"/>
-      <c r="C53" s="61"/>
-      <c r="D53" s="61"/>
-      <c r="E53" s="61"/>
+      <c r="A53" s="71"/>
+      <c r="B53" s="71"/>
+      <c r="C53" s="63"/>
+      <c r="D53" s="63"/>
+      <c r="E53" s="63"/>
       <c r="F53" s="52"/>
       <c r="G53" s="52"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="62"/>
-      <c r="B54" s="62"/>
-      <c r="C54" s="61"/>
-      <c r="D54" s="61"/>
-      <c r="E54" s="61"/>
+      <c r="A54" s="71"/>
+      <c r="B54" s="71"/>
+      <c r="C54" s="63"/>
+      <c r="D54" s="63"/>
+      <c r="E54" s="63"/>
       <c r="F54" s="52"/>
       <c r="G54" s="52"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="62"/>
-      <c r="B55" s="62"/>
-      <c r="C55" s="61"/>
-      <c r="D55" s="61"/>
-      <c r="E55" s="61"/>
+      <c r="A55" s="71"/>
+      <c r="B55" s="71"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="63"/>
+      <c r="E55" s="63"/>
       <c r="F55" s="52"/>
       <c r="G55" s="52"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="62"/>
-      <c r="B56" s="62"/>
-      <c r="C56" s="61"/>
-      <c r="D56" s="61"/>
-      <c r="E56" s="61"/>
+      <c r="A56" s="71"/>
+      <c r="B56" s="71"/>
+      <c r="C56" s="63"/>
+      <c r="D56" s="63"/>
+      <c r="E56" s="63"/>
       <c r="F56" s="52"/>
       <c r="G56" s="52"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="62"/>
-      <c r="B57" s="62"/>
-      <c r="C57" s="61"/>
-      <c r="D57" s="61"/>
-      <c r="E57" s="61"/>
+      <c r="A57" s="71"/>
+      <c r="B57" s="71"/>
+      <c r="C57" s="63"/>
+      <c r="D57" s="63"/>
+      <c r="E57" s="63"/>
       <c r="F57" s="52"/>
       <c r="G57" s="52"/>
     </row>
     <row r="58" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="62"/>
-      <c r="B58" s="62"/>
-      <c r="C58" s="61"/>
-      <c r="D58" s="61"/>
-      <c r="E58" s="61"/>
+      <c r="A58" s="71"/>
+      <c r="B58" s="71"/>
+      <c r="C58" s="63"/>
+      <c r="D58" s="63"/>
+      <c r="E58" s="63"/>
       <c r="F58" s="52"/>
       <c r="G58" s="52"/>
     </row>
     <row r="59" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="62"/>
-      <c r="B59" s="62"/>
+      <c r="A59" s="71"/>
+      <c r="B59" s="71"/>
       <c r="C59" s="30"/>
       <c r="D59" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="E59" s="61"/>
-      <c r="F59" s="63" t="s">
+      <c r="E59" s="63"/>
+      <c r="F59" s="64" t="s">
         <v>136</v>
       </c>
-      <c r="G59" s="64"/>
+      <c r="G59" s="65"/>
     </row>
     <row r="60" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="62"/>
-      <c r="B60" s="62"/>
+      <c r="A60" s="71"/>
+      <c r="B60" s="71"/>
       <c r="C60" s="14" t="s">
         <v>112</v>
       </c>
@@ -10251,13 +9204,13 @@
         <f>SUM(E10:E36)</f>
         <v>201</v>
       </c>
-      <c r="E60" s="61"/>
-      <c r="F60" s="65"/>
-      <c r="G60" s="66"/>
+      <c r="E60" s="63"/>
+      <c r="F60" s="66"/>
+      <c r="G60" s="67"/>
     </row>
     <row r="61" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="62"/>
-      <c r="B61" s="62"/>
+      <c r="A61" s="71"/>
+      <c r="B61" s="71"/>
       <c r="C61" s="14" t="s">
         <v>123</v>
       </c>
@@ -10265,13 +9218,13 @@
         <f>D60-D48</f>
         <v>164</v>
       </c>
-      <c r="E61" s="61"/>
-      <c r="F61" s="67"/>
-      <c r="G61" s="68"/>
+      <c r="E61" s="63"/>
+      <c r="F61" s="68"/>
+      <c r="G61" s="69"/>
     </row>
     <row r="62" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="62"/>
-      <c r="B62" s="62"/>
+      <c r="A62" s="71"/>
+      <c r="B62" s="71"/>
       <c r="C62" s="14" t="s">
         <v>120</v>
       </c>
@@ -10279,17 +9232,17 @@
         <f>D61-D49</f>
         <v>107</v>
       </c>
-      <c r="E62" s="61"/>
+      <c r="E62" s="63"/>
       <c r="F62" s="49" t="s">
         <v>124</v>
       </c>
       <c r="G62" s="50" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="62"/>
-      <c r="B63" s="62"/>
+      <c r="A63" s="71"/>
+      <c r="B63" s="71"/>
       <c r="C63" s="14" t="s">
         <v>122</v>
       </c>
@@ -10297,18 +9250,18 @@
         <f>D62-E50</f>
         <v>44</v>
       </c>
-      <c r="E63" s="61"/>
+      <c r="E63" s="63"/>
       <c r="F63" s="45" t="s">
         <v>115</v>
       </c>
       <c r="G63" s="43">
         <f>VLOOKUP(G62,C46:G51,3,FALSE)</f>
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="62"/>
-      <c r="B64" s="62"/>
+      <c r="A64" s="71"/>
+      <c r="B64" s="71"/>
       <c r="C64" s="14" t="s">
         <v>121</v>
       </c>
@@ -10316,98 +9269,98 @@
         <f>D51+F50-E51</f>
         <v>0</v>
       </c>
-      <c r="E64" s="61"/>
+      <c r="E64" s="63"/>
       <c r="F64" s="45" t="s">
         <v>117</v>
       </c>
       <c r="G64" s="43">
         <f>VLOOKUP(G62,C46:G51,2,FALSE)</f>
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="62"/>
-      <c r="B65" s="62"/>
-      <c r="C65" s="61"/>
-      <c r="D65" s="61"/>
-      <c r="E65" s="61"/>
-      <c r="F65" s="61"/>
-      <c r="G65" s="61"/>
+      <c r="A65" s="71"/>
+      <c r="B65" s="71"/>
+      <c r="C65" s="63"/>
+      <c r="D65" s="63"/>
+      <c r="E65" s="63"/>
+      <c r="F65" s="63"/>
+      <c r="G65" s="63"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="62"/>
-      <c r="B66" s="62"/>
-      <c r="C66" s="61"/>
-      <c r="D66" s="61"/>
-      <c r="E66" s="61"/>
-      <c r="F66" s="61"/>
-      <c r="G66" s="61"/>
+      <c r="A66" s="71"/>
+      <c r="B66" s="71"/>
+      <c r="C66" s="63"/>
+      <c r="D66" s="63"/>
+      <c r="E66" s="63"/>
+      <c r="F66" s="63"/>
+      <c r="G66" s="63"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="62"/>
-      <c r="B67" s="62"/>
-      <c r="C67" s="61"/>
-      <c r="D67" s="61"/>
-      <c r="E67" s="61"/>
-      <c r="F67" s="61"/>
-      <c r="G67" s="61"/>
+      <c r="A67" s="71"/>
+      <c r="B67" s="71"/>
+      <c r="C67" s="63"/>
+      <c r="D67" s="63"/>
+      <c r="E67" s="63"/>
+      <c r="F67" s="63"/>
+      <c r="G67" s="63"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="62"/>
-      <c r="B68" s="62"/>
-      <c r="C68" s="61"/>
-      <c r="D68" s="61"/>
-      <c r="E68" s="61"/>
-      <c r="F68" s="61"/>
-      <c r="G68" s="61"/>
+      <c r="A68" s="71"/>
+      <c r="B68" s="71"/>
+      <c r="C68" s="63"/>
+      <c r="D68" s="63"/>
+      <c r="E68" s="63"/>
+      <c r="F68" s="63"/>
+      <c r="G68" s="63"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="62"/>
-      <c r="B69" s="62"/>
-      <c r="C69" s="61"/>
-      <c r="D69" s="61"/>
-      <c r="E69" s="61"/>
-      <c r="F69" s="61"/>
-      <c r="G69" s="61"/>
+      <c r="A69" s="71"/>
+      <c r="B69" s="71"/>
+      <c r="C69" s="63"/>
+      <c r="D69" s="63"/>
+      <c r="E69" s="63"/>
+      <c r="F69" s="63"/>
+      <c r="G69" s="63"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B71" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="E59:E64"/>
+    <mergeCell ref="F59:G61"/>
     <mergeCell ref="C65:G69"/>
+    <mergeCell ref="A1:G8"/>
     <mergeCell ref="A37:B69"/>
-    <mergeCell ref="F59:G61"/>
-    <mergeCell ref="C52:E58"/>
-    <mergeCell ref="A1:G8"/>
-    <mergeCell ref="E59:E64"/>
     <mergeCell ref="C37:G45"/>
-    <mergeCell ref="F51:G51"/>
     <mergeCell ref="F46:G46"/>
     <mergeCell ref="F47:G47"/>
     <mergeCell ref="F48:G48"/>
     <mergeCell ref="F49:G49"/>
     <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="C52:E58"/>
   </mergeCells>
   <conditionalFormatting sqref="A10:D36 F10:G36">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>#REF!="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>#REF!=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="8">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira uma descrição do item nesta coluna" sqref="B9" xr:uid="{3E0CDA96-62DA-4783-91B0-EAD60F8F8A14}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o preço unitário de cada item nesta coluna" sqref="C9" xr:uid="{72914D10-8A28-40C0-9FE1-EE37279638B5}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira a quantidade em estoque de cada item nesta coluna" sqref="D9" xr:uid="{6399A917-1012-4753-A266-23A4E693DD3B}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Esse é um valor de estoque column._x000a__x000a_O valor de estoque de cada item é automaticamente calculado nesta coluna." sqref="E9" xr:uid="{6DA33C9F-E7EB-4EBB-BE05-900589138049}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nível de estoque de cada item nesta coluna" sqref="F9" xr:uid="{8FAF9DD4-C30E-4934-9B5E-7C6B02F23E75}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira quantos dias faltam para realizar nova encomenda de cada item nesta coluna" sqref="G9" xr:uid="{CBC61B02-1456-47C8-A9D5-E64F7EEDE2A3}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nome do item nesta coluna" sqref="A9" xr:uid="{4AEACA9D-41A6-4BE8-BD8B-AE83A899E5EE}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G62" xr:uid="{259A99CB-B18F-4E5F-9C4F-7B0E2CA304A4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G62" xr:uid="{48A427D4-E98B-4464-8932-C27C4F25EBEB}">
       <formula1>$C$48:$C$51</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nome do item nesta coluna" sqref="A9" xr:uid="{F68BE7A7-AEC5-4C2F-ADBE-A75174293901}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira quantos dias faltam para realizar nova encomenda de cada item nesta coluna" sqref="G9" xr:uid="{7B9C7BF5-5261-46AB-AB3D-17E3CF322AFA}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o nível de estoque de cada item nesta coluna" sqref="F9" xr:uid="{C4A02465-4662-40A3-BD6B-75874F44CCD7}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Esse é um valor de estoque column._x000a__x000a_O valor de estoque de cada item é automaticamente calculado nesta coluna." sqref="E9" xr:uid="{8D368F22-17EA-4D58-A7DC-08CCB36CCD50}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira a quantidade em estoque de cada item nesta coluna" sqref="D9" xr:uid="{FFB33C16-B029-4D4D-9A01-AC6077AC35F6}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira o preço unitário de cada item nesta coluna" sqref="C9" xr:uid="{650C0D00-0C81-483A-B470-9B922899F74C}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Insira uma descrição do item nesta coluna" sqref="B9" xr:uid="{D1F626B7-F27B-4554-BB65-289A9B6DD78C}"/>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -10418,51 +9371,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
-    <xsd:import namespace="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <xsd:import namespace="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <xsd:import namespace="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A729CFA7192B0F4AA60BE2DF65F4BC74" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c88fc727e37bcbeb6d3a40296a022323">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8497f9ae-9c71-438c-b553-1e6fe8b1acb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="77a4e7418373acf0c30a5fd0050b4a86" ns3:_="">
+    <xsd:import namespace="8497f9ae-9c71-438c-b553-1e6fe8b1acb0"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
-                <xsd:element ref="ns2:Status" minOccurs="0"/>
-                <xsd:element ref="ns2:Image" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:ImageTagsTaxHTField" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:Background" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDocTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -10470,173 +9392,33 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8497f9ae-9c71-438c-b553-1e6fe8b1acb0" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="20" nillable="true" ma:displayName="Unified Compliance Policy Properties" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties" ma:readOnly="false">
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="21" nillable="true" ma:displayName="Unified Compliance Policy UI Action" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction" ma:readOnly="false">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="Status" ma:index="2" nillable="true" ma:displayName="Status" ma:default="Not started" ma:format="Dropdown" ma:internalName="Status" ma:readOnly="false">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="Not started"/>
-          <xsd:enumeration value="In Progress"/>
-          <xsd:enumeration value="Completed"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Image" ma:index="3" nillable="true" ma:displayName="Image" ma:format="Image" ma:internalName="Image" ma:readOnly="false">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:URL">
-            <xsd:sequence>
-              <xsd:element name="Url" type="dms:ValidUrl" minOccurs="0" nillable="true"/>
-              <xsd:element name="Description" type="xsd:string" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceFastMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="10" nillable="true" ma:displayName="MediaServiceOCR" ma:hidden="true" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="_activity" ma:index="12" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="MediaServiceAutoTags" ma:hidden="true" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="12" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:hidden="true" ma:internalName="MediaServiceKeyPoints" ma:readOnly="false">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="ImageTagsTaxHTField" ma:index="25" nillable="true" ma:taxonomy="true" ma:internalName="ImageTagsTaxHTField" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e385fb40-52d4-4fae-9c5b-3e8ff8a5878e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="26" nillable="true" ma:displayName="Location" ma:hidden="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="27" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Background" ma:index="28" nillable="true" ma:displayName="Background" ma:default="0" ma:format="Dropdown" ma:internalName="Background">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Boolean"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="29" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDocTags" ma:index="30" nillable="true" ma:displayName="MediaServiceDocTags" ma:hidden="true" ma:internalName="MediaServiceDocTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="31" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSystemTags" ma:index="32" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="16c05727-aa75-4e4a-9b5f-8a80a1165891" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="14" nillable="true" ma:displayName="Shared With" ma:hidden="true" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="15" nillable="true" ma:displayName="Shared With Details" ma:hidden="true" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="230e9df3-be65-4c73-a93b-d1236ebd677e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3f6bfcbc-3db3-4ae6-bd76-326f0798ad28}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="16c05727-aa75-4e4a-9b5f-8a80a1165891">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -10648,8 +9430,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="1" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -10738,45 +9520,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+    <_activity xmlns="8497f9ae-9c71-438c-b553-1e6fe8b1acb0" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A83B3E02-9081-4283-A1B6-3FADACFC660C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84764C01-755B-4501-9893-DE1587D322EE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A3FC760-E629-409A-86BC-CC3C163C0ACB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="8497f9ae-9c71-438c-b553-1e6fe8b1acb0"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -10787,21 +9555,26 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A83B3E02-9081-4283-A1B6-3FADACFC660C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E347ADB8-BE75-4F14-ADF9-E64D4A3FD476}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8497f9ae-9c71-438c-b553-1e6fe8b1acb0"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>